<commit_message>
Initial submission: data, notebooks, summary, figures
</commit_message>
<xml_diff>
--- a/output/app_updates.xlsx
+++ b/output/app_updates.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24990" windowHeight="14835" activeTab="1"/>
+    <workbookView windowHeight="18360" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1172,7 +1172,7 @@
     <t>Date: May 7, 2026</t>
   </si>
   <si>
-    <t>Repository: https://github.com/lcy432/wliura-app-updates  (placeholder — replace with actual URL before submission)</t>
+    <t>Repository: https://github.com/lcy432/release-notes-llm-classifier</t>
   </si>
   <si>
     <t>Dataset: 85 rows after dedup (one per app × platform × version), covering 10 apps from 2008-07-11 to 2026-05-06.</t>

</xml_diff>